<commit_message>
feat: update statuses in excel
</commit_message>
<xml_diff>
--- a/CDOP Enumerated Values Lists.xlsx
+++ b/CDOP Enumerated Values Lists.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rockmtnins-my.sharepoint.com/personal/sebastian_weeks_rmi_org/Documents/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sylvera/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{05BEAEA2-6A2F-4741-AE99-4729EDC813A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A107595E-E8AE-4385-A26A-F5427270776A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D9CD72BC-0048-E34B-8951-ECDC5031725B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{6157C829-B9E8-47C5-B94D-577BB9DC27B4}"/>
+    <workbookView xWindow="1600" yWindow="-18140" windowWidth="29400" windowHeight="16600" xr2:uid="{6157C829-B9E8-47C5-B94D-577BB9DC27B4}"/>
   </bookViews>
   <sheets>
     <sheet name="Enumerated Values Lists" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1395" uniqueCount="1354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1396" uniqueCount="1354">
   <si>
     <t>Enumerated Values List</t>
   </si>
@@ -4082,22 +4082,22 @@
     <t>issuance status</t>
   </si>
   <si>
-    <t>Verified</t>
-  </si>
-  <si>
-    <t>Pending Issuance</t>
-  </si>
-  <si>
-    <t>Issuing</t>
-  </si>
-  <si>
-    <t>Pre-issuance</t>
-  </si>
-  <si>
-    <t>Failed</t>
-  </si>
-  <si>
     <t>Complete</t>
+  </si>
+  <si>
+    <t>Project design</t>
+  </si>
+  <si>
+    <t>Validation</t>
+  </si>
+  <si>
+    <t>First verification</t>
+  </si>
+  <si>
+    <t>Verified and issuing</t>
+  </si>
+  <si>
+    <t>Initial assessment and feasability</t>
   </si>
 </sst>
 </file>
@@ -4574,15 +4574,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B85F238-80B8-43F8-AABF-7B9427088CCA}">
   <dimension ref="A1:AW499"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="27" max="27" width="11.08984375" customWidth="1"/>
+    <col min="27" max="27" width="11.1640625" customWidth="1"/>
     <col min="45" max="46" width="12" customWidth="1"/>
-    <col min="47" max="48" width="14.7265625" customWidth="1"/>
-    <col min="49" max="49" width="16.90625" customWidth="1"/>
+    <col min="47" max="48" width="14.6640625" customWidth="1"/>
+    <col min="49" max="49" width="16.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -4605,7 +4605,7 @@
       <c r="R1" s="4"/>
       <c r="S1" s="4"/>
     </row>
-    <row r="2" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
@@ -4626,7 +4626,7 @@
       <c r="R2" s="4"/>
       <c r="S2" s="4"/>
     </row>
-    <row r="3" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -4725,7 +4725,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="4" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>11</v>
       </c>
@@ -4815,10 +4815,10 @@
         <v>614</v>
       </c>
       <c r="AW4" s="4" t="s">
-        <v>1348</v>
-      </c>
-    </row>
-    <row r="5" spans="1:49" x14ac:dyDescent="0.35">
+        <v>1353</v>
+      </c>
+    </row>
+    <row r="5" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
         <v>21</v>
       </c>
@@ -4905,7 +4905,7 @@
         <v>1349</v>
       </c>
     </row>
-    <row r="6" spans="1:49" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:49" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>29</v>
       </c>
@@ -4992,7 +4992,7 @@
         <v>1350</v>
       </c>
     </row>
-    <row r="7" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
         <v>36</v>
       </c>
@@ -5069,10 +5069,10 @@
         <v>649</v>
       </c>
       <c r="AW7" s="4" t="s">
-        <v>1351</v>
-      </c>
-    </row>
-    <row r="8" spans="1:49" x14ac:dyDescent="0.35">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="8" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
         <v>42</v>
       </c>
@@ -5145,10 +5145,10 @@
         <v>659</v>
       </c>
       <c r="AW8" s="4" t="s">
-        <v>1352</v>
-      </c>
-    </row>
-    <row r="9" spans="1:49" x14ac:dyDescent="0.35">
+        <v>1351</v>
+      </c>
+    </row>
+    <row r="9" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
         <v>48</v>
       </c>
@@ -5224,10 +5224,10 @@
         <v>668</v>
       </c>
       <c r="AW9" s="4" t="s">
-        <v>1353</v>
-      </c>
-    </row>
-    <row r="10" spans="1:49" x14ac:dyDescent="0.35">
+        <v>1352</v>
+      </c>
+    </row>
+    <row r="10" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
         <v>54</v>
       </c>
@@ -5291,8 +5291,11 @@
       <c r="AU10" t="s">
         <v>677</v>
       </c>
-    </row>
-    <row r="11" spans="1:49" x14ac:dyDescent="0.35">
+      <c r="AW10" s="4" t="s">
+        <v>1348</v>
+      </c>
+    </row>
+    <row r="11" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A11" s="8" t="s">
         <v>60</v>
       </c>
@@ -5358,7 +5361,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="12" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
         <v>66</v>
       </c>
@@ -5420,7 +5423,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="13" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A13" s="8" t="s">
         <v>71</v>
       </c>
@@ -5484,7 +5487,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="14" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
         <v>76</v>
       </c>
@@ -5549,7 +5552,7 @@
         <v>708</v>
       </c>
     </row>
-    <row r="15" spans="1:49" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A15" s="8" t="s">
         <v>81</v>
       </c>
@@ -5607,8 +5610,9 @@
       <c r="AU15" t="s">
         <v>716</v>
       </c>
-    </row>
-    <row r="16" spans="1:49" x14ac:dyDescent="0.35">
+      <c r="AW15" s="4"/>
+    </row>
+    <row r="16" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
         <v>86</v>
       </c>
@@ -5669,7 +5673,7 @@
         <v>723</v>
       </c>
     </row>
-    <row r="17" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:47" x14ac:dyDescent="0.2">
       <c r="A17" s="8" t="s">
         <v>91</v>
       </c>
@@ -5729,7 +5733,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="18" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:47" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
         <v>96</v>
       </c>
@@ -5789,7 +5793,7 @@
         <v>735</v>
       </c>
     </row>
-    <row r="19" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:47" x14ac:dyDescent="0.2">
       <c r="A19" s="8" t="s">
         <v>100</v>
       </c>
@@ -5848,7 +5852,7 @@
         <v>742</v>
       </c>
     </row>
-    <row r="20" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:47" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
         <v>105</v>
       </c>
@@ -5907,7 +5911,7 @@
         <v>749</v>
       </c>
     </row>
-    <row r="21" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:47" x14ac:dyDescent="0.2">
       <c r="A21" s="8" t="s">
         <v>109</v>
       </c>
@@ -5965,7 +5969,7 @@
         <v>755</v>
       </c>
     </row>
-    <row r="22" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:47" x14ac:dyDescent="0.2">
       <c r="A22" s="5" t="s">
         <v>113</v>
       </c>
@@ -6015,7 +6019,7 @@
         <v>766</v>
       </c>
     </row>
-    <row r="23" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:47" x14ac:dyDescent="0.2">
       <c r="A23" s="8" t="s">
         <v>117</v>
       </c>
@@ -6061,7 +6065,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="24" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:47" x14ac:dyDescent="0.2">
       <c r="A24" s="5" t="s">
         <v>121</v>
       </c>
@@ -6108,7 +6112,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="25" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:47" x14ac:dyDescent="0.2">
       <c r="A25" s="8" t="s">
         <v>125</v>
       </c>
@@ -6156,7 +6160,7 @@
         <v>780</v>
       </c>
     </row>
-    <row r="26" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:47" x14ac:dyDescent="0.2">
       <c r="A26" s="5" t="s">
         <v>129</v>
       </c>
@@ -6199,7 +6203,7 @@
         <v>784</v>
       </c>
     </row>
-    <row r="27" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:47" x14ac:dyDescent="0.2">
       <c r="A27" s="8" t="s">
         <v>133</v>
       </c>
@@ -6242,7 +6246,7 @@
         <v>788</v>
       </c>
     </row>
-    <row r="28" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:47" x14ac:dyDescent="0.2">
       <c r="A28" s="5" t="s">
         <v>137</v>
       </c>
@@ -6284,7 +6288,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="29" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:47" x14ac:dyDescent="0.2">
       <c r="A29" s="8" t="s">
         <v>141</v>
       </c>
@@ -6327,7 +6331,7 @@
         <v>795</v>
       </c>
     </row>
-    <row r="30" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:47" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
         <v>145</v>
       </c>
@@ -6371,7 +6375,7 @@
         <v>798</v>
       </c>
     </row>
-    <row r="31" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:47" x14ac:dyDescent="0.2">
       <c r="A31" s="8" t="s">
         <v>149</v>
       </c>
@@ -6414,7 +6418,7 @@
         <v>801</v>
       </c>
     </row>
-    <row r="32" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:47" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
         <v>153</v>
       </c>
@@ -6457,7 +6461,7 @@
         <v>804</v>
       </c>
     </row>
-    <row r="33" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A33" s="8" t="s">
         <v>157</v>
       </c>
@@ -6501,7 +6505,7 @@
         <v>807</v>
       </c>
     </row>
-    <row r="34" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A34" s="5" t="s">
         <v>161</v>
       </c>
@@ -6545,7 +6549,7 @@
         <v>811</v>
       </c>
     </row>
-    <row r="35" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A35" s="8" t="s">
         <v>165</v>
       </c>
@@ -6585,7 +6589,7 @@
         <v>814</v>
       </c>
     </row>
-    <row r="36" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
         <v>167</v>
       </c>
@@ -6623,7 +6627,7 @@
         <v>817</v>
       </c>
     </row>
-    <row r="37" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A37" s="8" t="s">
         <v>169</v>
       </c>
@@ -6663,7 +6667,7 @@
         <v>821</v>
       </c>
     </row>
-    <row r="38" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A38" s="5" t="s">
         <v>171</v>
       </c>
@@ -6702,7 +6706,7 @@
         <v>824</v>
       </c>
     </row>
-    <row r="39" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A39" s="8" t="s">
         <v>173</v>
       </c>
@@ -6738,7 +6742,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="40" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A40" s="5" t="s">
         <v>175</v>
       </c>
@@ -6774,7 +6778,7 @@
         <v>829</v>
       </c>
     </row>
-    <row r="41" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A41" s="8" t="s">
         <v>177</v>
       </c>
@@ -6810,7 +6814,7 @@
         <v>831</v>
       </c>
     </row>
-    <row r="42" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A42" s="5" t="s">
         <v>179</v>
       </c>
@@ -6845,7 +6849,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="43" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A43" s="8" t="s">
         <v>181</v>
       </c>
@@ -6881,7 +6885,7 @@
         <v>836</v>
       </c>
     </row>
-    <row r="44" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A44" s="5" t="s">
         <v>183</v>
       </c>
@@ -6917,7 +6921,7 @@
         <v>838</v>
       </c>
     </row>
-    <row r="45" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A45" s="8" t="s">
         <v>185</v>
       </c>
@@ -6952,7 +6956,7 @@
         <v>841</v>
       </c>
     </row>
-    <row r="46" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A46" s="5" t="s">
         <v>187</v>
       </c>
@@ -6988,7 +6992,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="47" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A47" s="8" t="s">
         <v>189</v>
       </c>
@@ -7020,7 +7024,7 @@
         <v>845</v>
       </c>
     </row>
-    <row r="48" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A48" s="5" t="s">
         <v>191</v>
       </c>
@@ -7052,7 +7056,7 @@
         <v>847</v>
       </c>
     </row>
-    <row r="49" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A49" s="8" t="s">
         <v>193</v>
       </c>
@@ -7084,7 +7088,7 @@
         <v>849</v>
       </c>
     </row>
-    <row r="50" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A50" s="5" t="s">
         <v>195</v>
       </c>
@@ -7116,7 +7120,7 @@
         <v>851</v>
       </c>
     </row>
-    <row r="51" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A51" s="8" t="s">
         <v>197</v>
       </c>
@@ -7148,7 +7152,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="52" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A52" s="5" t="s">
         <v>199</v>
       </c>
@@ -7180,7 +7184,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="53" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A53" s="8" t="s">
         <v>201</v>
       </c>
@@ -7212,7 +7216,7 @@
         <v>857</v>
       </c>
     </row>
-    <row r="54" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A54" s="5" t="s">
         <v>203</v>
       </c>
@@ -7244,7 +7248,7 @@
         <v>859</v>
       </c>
     </row>
-    <row r="55" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A55" s="8" t="s">
         <v>205</v>
       </c>
@@ -7276,7 +7280,7 @@
         <v>861</v>
       </c>
     </row>
-    <row r="56" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A56" s="5" t="s">
         <v>207</v>
       </c>
@@ -7308,7 +7312,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="57" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A57" s="8" t="s">
         <v>209</v>
       </c>
@@ -7340,7 +7344,7 @@
         <v>865</v>
       </c>
     </row>
-    <row r="58" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A58" s="5" t="s">
         <v>211</v>
       </c>
@@ -7372,7 +7376,7 @@
         <v>867</v>
       </c>
     </row>
-    <row r="59" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A59" s="8" t="s">
         <v>213</v>
       </c>
@@ -7404,7 +7408,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="60" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A60" s="5" t="s">
         <v>215</v>
       </c>
@@ -7436,7 +7440,7 @@
         <v>871</v>
       </c>
     </row>
-    <row r="61" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A61" s="8" t="s">
         <v>217</v>
       </c>
@@ -7468,7 +7472,7 @@
         <v>873</v>
       </c>
     </row>
-    <row r="62" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A62" s="5" t="s">
         <v>219</v>
       </c>
@@ -7500,7 +7504,7 @@
         <v>875</v>
       </c>
     </row>
-    <row r="63" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A63" s="8" t="s">
         <v>221</v>
       </c>
@@ -7532,7 +7536,7 @@
         <v>877</v>
       </c>
     </row>
-    <row r="64" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A64" s="5" t="s">
         <v>223</v>
       </c>
@@ -7564,7 +7568,7 @@
         <v>879</v>
       </c>
     </row>
-    <row r="65" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A65" s="8" t="s">
         <v>225</v>
       </c>
@@ -7596,7 +7600,7 @@
         <v>881</v>
       </c>
     </row>
-    <row r="66" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A66" s="5" t="s">
         <v>227</v>
       </c>
@@ -7628,7 +7632,7 @@
         <v>883</v>
       </c>
     </row>
-    <row r="67" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A67" s="8" t="s">
         <v>229</v>
       </c>
@@ -7660,7 +7664,7 @@
         <v>885</v>
       </c>
     </row>
-    <row r="68" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A68" s="5" t="s">
         <v>231</v>
       </c>
@@ -7692,7 +7696,7 @@
         <v>887</v>
       </c>
     </row>
-    <row r="69" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A69" s="8" t="s">
         <v>233</v>
       </c>
@@ -7724,7 +7728,7 @@
         <v>889</v>
       </c>
     </row>
-    <row r="70" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A70" s="5" t="s">
         <v>235</v>
       </c>
@@ -7756,7 +7760,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="71" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A71" s="8" t="s">
         <v>237</v>
       </c>
@@ -7788,7 +7792,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="72" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A72" s="5" t="s">
         <v>239</v>
       </c>
@@ -7820,7 +7824,7 @@
         <v>895</v>
       </c>
     </row>
-    <row r="73" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A73" s="8" t="s">
         <v>241</v>
       </c>
@@ -7852,7 +7856,7 @@
         <v>897</v>
       </c>
     </row>
-    <row r="74" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A74" s="5" t="s">
         <v>243</v>
       </c>
@@ -7884,7 +7888,7 @@
         <v>899</v>
       </c>
     </row>
-    <row r="75" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A75" s="8" t="s">
         <v>245</v>
       </c>
@@ -7916,7 +7920,7 @@
         <v>901</v>
       </c>
     </row>
-    <row r="76" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A76" s="5" t="s">
         <v>247</v>
       </c>
@@ -7948,7 +7952,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="77" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A77" s="8" t="s">
         <v>249</v>
       </c>
@@ -7980,7 +7984,7 @@
         <v>905</v>
       </c>
     </row>
-    <row r="78" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A78" s="5" t="s">
         <v>251</v>
       </c>
@@ -8012,7 +8016,7 @@
         <v>907</v>
       </c>
     </row>
-    <row r="79" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A79" s="8" t="s">
         <v>253</v>
       </c>
@@ -8044,7 +8048,7 @@
         <v>909</v>
       </c>
     </row>
-    <row r="80" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A80" s="5" t="s">
         <v>255</v>
       </c>
@@ -8076,7 +8080,7 @@
         <v>911</v>
       </c>
     </row>
-    <row r="81" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A81" s="8" t="s">
         <v>257</v>
       </c>
@@ -8108,7 +8112,7 @@
         <v>913</v>
       </c>
     </row>
-    <row r="82" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A82" s="5" t="s">
         <v>259</v>
       </c>
@@ -8140,7 +8144,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="83" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A83" s="8" t="s">
         <v>261</v>
       </c>
@@ -8172,7 +8176,7 @@
         <v>917</v>
       </c>
     </row>
-    <row r="84" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A84" s="5" t="s">
         <v>263</v>
       </c>
@@ -8204,7 +8208,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="85" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A85" s="8" t="s">
         <v>265</v>
       </c>
@@ -8236,7 +8240,7 @@
         <v>921</v>
       </c>
     </row>
-    <row r="86" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A86" s="5" t="s">
         <v>267</v>
       </c>
@@ -8268,7 +8272,7 @@
         <v>923</v>
       </c>
     </row>
-    <row r="87" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A87" s="8" t="s">
         <v>269</v>
       </c>
@@ -8300,7 +8304,7 @@
         <v>925</v>
       </c>
     </row>
-    <row r="88" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A88" s="5" t="s">
         <v>271</v>
       </c>
@@ -8332,7 +8336,7 @@
         <v>927</v>
       </c>
     </row>
-    <row r="89" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A89" s="8" t="s">
         <v>273</v>
       </c>
@@ -8364,7 +8368,7 @@
         <v>929</v>
       </c>
     </row>
-    <row r="90" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A90" s="5" t="s">
         <v>275</v>
       </c>
@@ -8396,7 +8400,7 @@
         <v>931</v>
       </c>
     </row>
-    <row r="91" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A91" s="8" t="s">
         <v>277</v>
       </c>
@@ -8424,7 +8428,7 @@
         <v>932</v>
       </c>
     </row>
-    <row r="92" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A92" s="5" t="s">
         <v>279</v>
       </c>
@@ -8452,7 +8456,7 @@
         <v>933</v>
       </c>
     </row>
-    <row r="93" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A93" s="8" t="s">
         <v>281</v>
       </c>
@@ -8480,7 +8484,7 @@
         <v>934</v>
       </c>
     </row>
-    <row r="94" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A94" s="5" t="s">
         <v>283</v>
       </c>
@@ -8508,7 +8512,7 @@
         <v>935</v>
       </c>
     </row>
-    <row r="95" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A95" s="8" t="s">
         <v>285</v>
       </c>
@@ -8536,7 +8540,7 @@
         <v>936</v>
       </c>
     </row>
-    <row r="96" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A96" s="5" t="s">
         <v>287</v>
       </c>
@@ -8564,7 +8568,7 @@
         <v>937</v>
       </c>
     </row>
-    <row r="97" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A97" s="8" t="s">
         <v>289</v>
       </c>
@@ -8592,7 +8596,7 @@
         <v>938</v>
       </c>
     </row>
-    <row r="98" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A98" s="5" t="s">
         <v>291</v>
       </c>
@@ -8620,7 +8624,7 @@
         <v>939</v>
       </c>
     </row>
-    <row r="99" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A99" s="8" t="s">
         <v>293</v>
       </c>
@@ -8648,7 +8652,7 @@
         <v>940</v>
       </c>
     </row>
-    <row r="100" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A100" s="5" t="s">
         <v>295</v>
       </c>
@@ -8676,7 +8680,7 @@
         <v>941</v>
       </c>
     </row>
-    <row r="101" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A101" s="8" t="s">
         <v>297</v>
       </c>
@@ -8704,7 +8708,7 @@
         <v>942</v>
       </c>
     </row>
-    <row r="102" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A102" s="5" t="s">
         <v>299</v>
       </c>
@@ -8732,7 +8736,7 @@
         <v>943</v>
       </c>
     </row>
-    <row r="103" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A103" s="8" t="s">
         <v>301</v>
       </c>
@@ -8760,7 +8764,7 @@
         <v>944</v>
       </c>
     </row>
-    <row r="104" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A104" s="5" t="s">
         <v>303</v>
       </c>
@@ -8788,7 +8792,7 @@
         <v>945</v>
       </c>
     </row>
-    <row r="105" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A105" s="8" t="s">
         <v>305</v>
       </c>
@@ -8816,7 +8820,7 @@
         <v>946</v>
       </c>
     </row>
-    <row r="106" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A106" s="5" t="s">
         <v>307</v>
       </c>
@@ -8844,7 +8848,7 @@
         <v>947</v>
       </c>
     </row>
-    <row r="107" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A107" s="8" t="s">
         <v>309</v>
       </c>
@@ -8872,7 +8876,7 @@
         <v>948</v>
       </c>
     </row>
-    <row r="108" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A108" s="5" t="s">
         <v>311</v>
       </c>
@@ -8900,7 +8904,7 @@
         <v>949</v>
       </c>
     </row>
-    <row r="109" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A109" s="8" t="s">
         <v>313</v>
       </c>
@@ -8928,7 +8932,7 @@
         <v>950</v>
       </c>
     </row>
-    <row r="110" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A110" s="5" t="s">
         <v>315</v>
       </c>
@@ -8956,7 +8960,7 @@
         <v>951</v>
       </c>
     </row>
-    <row r="111" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A111" s="8" t="s">
         <v>317</v>
       </c>
@@ -8984,7 +8988,7 @@
         <v>952</v>
       </c>
     </row>
-    <row r="112" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A112" s="5" t="s">
         <v>319</v>
       </c>
@@ -9012,7 +9016,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="113" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A113" s="8" t="s">
         <v>321</v>
       </c>
@@ -9040,7 +9044,7 @@
         <v>954</v>
       </c>
     </row>
-    <row r="114" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A114" s="5" t="s">
         <v>323</v>
       </c>
@@ -9068,7 +9072,7 @@
         <v>955</v>
       </c>
     </row>
-    <row r="115" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A115" s="8" t="s">
         <v>325</v>
       </c>
@@ -9096,7 +9100,7 @@
         <v>956</v>
       </c>
     </row>
-    <row r="116" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A116" s="5" t="s">
         <v>327</v>
       </c>
@@ -9124,7 +9128,7 @@
         <v>957</v>
       </c>
     </row>
-    <row r="117" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A117" s="8" t="s">
         <v>329</v>
       </c>
@@ -9152,7 +9156,7 @@
         <v>958</v>
       </c>
     </row>
-    <row r="118" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A118" s="5" t="s">
         <v>331</v>
       </c>
@@ -9180,7 +9184,7 @@
         <v>959</v>
       </c>
     </row>
-    <row r="119" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A119" s="8" t="s">
         <v>333</v>
       </c>
@@ -9208,7 +9212,7 @@
         <v>960</v>
       </c>
     </row>
-    <row r="120" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A120" s="5" t="s">
         <v>335</v>
       </c>
@@ -9236,7 +9240,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="121" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A121" s="8" t="s">
         <v>337</v>
       </c>
@@ -9264,7 +9268,7 @@
         <v>962</v>
       </c>
     </row>
-    <row r="122" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A122" s="5" t="s">
         <v>339</v>
       </c>
@@ -9292,7 +9296,7 @@
         <v>963</v>
       </c>
     </row>
-    <row r="123" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A123" s="8" t="s">
         <v>341</v>
       </c>
@@ -9320,7 +9324,7 @@
         <v>964</v>
       </c>
     </row>
-    <row r="124" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A124" s="5" t="s">
         <v>343</v>
       </c>
@@ -9348,7 +9352,7 @@
         <v>965</v>
       </c>
     </row>
-    <row r="125" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A125" s="8" t="s">
         <v>345</v>
       </c>
@@ -9376,7 +9380,7 @@
         <v>966</v>
       </c>
     </row>
-    <row r="126" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A126" s="5" t="s">
         <v>347</v>
       </c>
@@ -9404,7 +9408,7 @@
         <v>967</v>
       </c>
     </row>
-    <row r="127" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A127" s="8" t="s">
         <v>349</v>
       </c>
@@ -9432,7 +9436,7 @@
         <v>968</v>
       </c>
     </row>
-    <row r="128" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A128" s="5" t="s">
         <v>351</v>
       </c>
@@ -9460,7 +9464,7 @@
         <v>969</v>
       </c>
     </row>
-    <row r="129" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A129" s="8" t="s">
         <v>353</v>
       </c>
@@ -9488,7 +9492,7 @@
         <v>970</v>
       </c>
     </row>
-    <row r="130" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A130" s="5" t="s">
         <v>355</v>
       </c>
@@ -9516,7 +9520,7 @@
         <v>971</v>
       </c>
     </row>
-    <row r="131" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A131" s="8" t="s">
         <v>357</v>
       </c>
@@ -9544,7 +9548,7 @@
         <v>972</v>
       </c>
     </row>
-    <row r="132" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A132" s="5" t="s">
         <v>359</v>
       </c>
@@ -9572,7 +9576,7 @@
         <v>973</v>
       </c>
     </row>
-    <row r="133" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A133" s="8" t="s">
         <v>361</v>
       </c>
@@ -9600,7 +9604,7 @@
         <v>974</v>
       </c>
     </row>
-    <row r="134" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A134" s="5" t="s">
         <v>363</v>
       </c>
@@ -9628,7 +9632,7 @@
         <v>975</v>
       </c>
     </row>
-    <row r="135" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A135" s="8" t="s">
         <v>365</v>
       </c>
@@ -9656,7 +9660,7 @@
         <v>976</v>
       </c>
     </row>
-    <row r="136" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A136" s="5" t="s">
         <v>367</v>
       </c>
@@ -9684,7 +9688,7 @@
         <v>977</v>
       </c>
     </row>
-    <row r="137" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A137" s="8" t="s">
         <v>369</v>
       </c>
@@ -9712,7 +9716,7 @@
         <v>978</v>
       </c>
     </row>
-    <row r="138" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A138" s="5" t="s">
         <v>371</v>
       </c>
@@ -9740,7 +9744,7 @@
         <v>979</v>
       </c>
     </row>
-    <row r="139" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A139" s="8" t="s">
         <v>373</v>
       </c>
@@ -9768,7 +9772,7 @@
         <v>980</v>
       </c>
     </row>
-    <row r="140" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A140" s="5" t="s">
         <v>375</v>
       </c>
@@ -9796,7 +9800,7 @@
         <v>981</v>
       </c>
     </row>
-    <row r="141" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A141" s="8" t="s">
         <v>377</v>
       </c>
@@ -9824,7 +9828,7 @@
         <v>982</v>
       </c>
     </row>
-    <row r="142" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A142" s="5" t="s">
         <v>379</v>
       </c>
@@ -9852,7 +9856,7 @@
         <v>983</v>
       </c>
     </row>
-    <row r="143" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A143" s="8" t="s">
         <v>381</v>
       </c>
@@ -9880,7 +9884,7 @@
         <v>984</v>
       </c>
     </row>
-    <row r="144" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A144" s="5" t="s">
         <v>383</v>
       </c>
@@ -9908,7 +9912,7 @@
         <v>985</v>
       </c>
     </row>
-    <row r="145" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A145" s="8" t="s">
         <v>385</v>
       </c>
@@ -9936,7 +9940,7 @@
         <v>986</v>
       </c>
     </row>
-    <row r="146" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A146" s="5" t="s">
         <v>387</v>
       </c>
@@ -9964,7 +9968,7 @@
         <v>987</v>
       </c>
     </row>
-    <row r="147" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A147" s="8" t="s">
         <v>389</v>
       </c>
@@ -9992,7 +9996,7 @@
         <v>988</v>
       </c>
     </row>
-    <row r="148" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A148" s="5" t="s">
         <v>391</v>
       </c>
@@ -10020,7 +10024,7 @@
         <v>989</v>
       </c>
     </row>
-    <row r="149" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A149" s="8" t="s">
         <v>393</v>
       </c>
@@ -10048,7 +10052,7 @@
         <v>990</v>
       </c>
     </row>
-    <row r="150" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A150" s="5" t="s">
         <v>395</v>
       </c>
@@ -10076,7 +10080,7 @@
         <v>991</v>
       </c>
     </row>
-    <row r="151" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A151" s="8" t="s">
         <v>397</v>
       </c>
@@ -10104,7 +10108,7 @@
         <v>992</v>
       </c>
     </row>
-    <row r="152" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A152" s="5" t="s">
         <v>399</v>
       </c>
@@ -10132,7 +10136,7 @@
         <v>993</v>
       </c>
     </row>
-    <row r="153" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A153" s="8" t="s">
         <v>401</v>
       </c>
@@ -10160,7 +10164,7 @@
         <v>994</v>
       </c>
     </row>
-    <row r="154" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A154" s="5" t="s">
         <v>403</v>
       </c>
@@ -10188,7 +10192,7 @@
         <v>995</v>
       </c>
     </row>
-    <row r="155" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A155" s="8" t="s">
         <v>405</v>
       </c>
@@ -10216,7 +10220,7 @@
         <v>996</v>
       </c>
     </row>
-    <row r="156" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A156" s="5" t="s">
         <v>407</v>
       </c>
@@ -10244,7 +10248,7 @@
         <v>997</v>
       </c>
     </row>
-    <row r="157" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A157" s="8" t="s">
         <v>409</v>
       </c>
@@ -10272,7 +10276,7 @@
         <v>998</v>
       </c>
     </row>
-    <row r="158" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A158" s="5" t="s">
         <v>411</v>
       </c>
@@ -10300,7 +10304,7 @@
         <v>999</v>
       </c>
     </row>
-    <row r="159" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A159" s="8" t="s">
         <v>413</v>
       </c>
@@ -10328,7 +10332,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="160" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A160" s="5" t="s">
         <v>415</v>
       </c>
@@ -10356,7 +10360,7 @@
         <v>1001</v>
       </c>
     </row>
-    <row r="161" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A161" s="8" t="s">
         <v>417</v>
       </c>
@@ -10384,7 +10388,7 @@
         <v>1002</v>
       </c>
     </row>
-    <row r="162" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A162" s="5" t="s">
         <v>419</v>
       </c>
@@ -10412,7 +10416,7 @@
         <v>1003</v>
       </c>
     </row>
-    <row r="163" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A163" s="8" t="s">
         <v>421</v>
       </c>
@@ -10440,7 +10444,7 @@
         <v>1004</v>
       </c>
     </row>
-    <row r="164" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A164" s="5" t="s">
         <v>423</v>
       </c>
@@ -10468,7 +10472,7 @@
         <v>1005</v>
       </c>
     </row>
-    <row r="165" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A165" s="8" t="s">
         <v>425</v>
       </c>
@@ -10496,7 +10500,7 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="166" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A166" s="5" t="s">
         <v>427</v>
       </c>
@@ -10524,7 +10528,7 @@
         <v>1007</v>
       </c>
     </row>
-    <row r="167" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A167" s="8" t="s">
         <v>429</v>
       </c>
@@ -10552,7 +10556,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="168" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A168" s="5" t="s">
         <v>431</v>
       </c>
@@ -10580,7 +10584,7 @@
         <v>1009</v>
       </c>
     </row>
-    <row r="169" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A169" s="8" t="s">
         <v>433</v>
       </c>
@@ -10608,7 +10612,7 @@
         <v>1010</v>
       </c>
     </row>
-    <row r="170" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A170" s="5" t="s">
         <v>435</v>
       </c>
@@ -10636,7 +10640,7 @@
         <v>1011</v>
       </c>
     </row>
-    <row r="171" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A171" s="8" t="s">
         <v>437</v>
       </c>
@@ -10664,7 +10668,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="172" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A172" s="5" t="s">
         <v>439</v>
       </c>
@@ -10692,7 +10696,7 @@
         <v>1013</v>
       </c>
     </row>
-    <row r="173" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A173" s="8" t="s">
         <v>441</v>
       </c>
@@ -10720,7 +10724,7 @@
         <v>1014</v>
       </c>
     </row>
-    <row r="174" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A174" s="5" t="s">
         <v>443</v>
       </c>
@@ -10748,7 +10752,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="175" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A175" s="8" t="s">
         <v>445</v>
       </c>
@@ -10776,7 +10780,7 @@
         <v>1016</v>
       </c>
     </row>
-    <row r="176" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A176" s="5" t="s">
         <v>447</v>
       </c>
@@ -10804,7 +10808,7 @@
         <v>1017</v>
       </c>
     </row>
-    <row r="177" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A177" s="8" t="s">
         <v>449</v>
       </c>
@@ -10832,7 +10836,7 @@
         <v>1018</v>
       </c>
     </row>
-    <row r="178" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A178" s="5" t="s">
         <v>451</v>
       </c>
@@ -10860,7 +10864,7 @@
         <v>1019</v>
       </c>
     </row>
-    <row r="179" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A179" s="8" t="s">
         <v>453</v>
       </c>
@@ -10888,7 +10892,7 @@
         <v>1020</v>
       </c>
     </row>
-    <row r="180" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A180" s="5" t="s">
         <v>455</v>
       </c>
@@ -10916,7 +10920,7 @@
         <v>1021</v>
       </c>
     </row>
-    <row r="181" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A181" s="8" t="s">
         <v>457</v>
       </c>
@@ -10944,7 +10948,7 @@
         <v>1022</v>
       </c>
     </row>
-    <row r="182" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A182" s="5" t="s">
         <v>459</v>
       </c>
@@ -10972,7 +10976,7 @@
         <v>1023</v>
       </c>
     </row>
-    <row r="183" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A183" s="8" t="s">
         <v>461</v>
       </c>
@@ -11000,7 +11004,7 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="184" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A184" s="5" t="s">
         <v>463</v>
       </c>
@@ -11028,7 +11032,7 @@
         <v>1025</v>
       </c>
     </row>
-    <row r="185" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A185" s="8" t="s">
         <v>465</v>
       </c>
@@ -11056,7 +11060,7 @@
         <v>1026</v>
       </c>
     </row>
-    <row r="186" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A186" s="5" t="s">
         <v>467</v>
       </c>
@@ -11084,7 +11088,7 @@
         <v>1027</v>
       </c>
     </row>
-    <row r="187" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A187" s="8" t="s">
         <v>469</v>
       </c>
@@ -11112,7 +11116,7 @@
         <v>1028</v>
       </c>
     </row>
-    <row r="188" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A188" s="5" t="s">
         <v>471</v>
       </c>
@@ -11140,7 +11144,7 @@
         <v>1029</v>
       </c>
     </row>
-    <row r="189" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A189" s="8" t="s">
         <v>473</v>
       </c>
@@ -11168,7 +11172,7 @@
         <v>1030</v>
       </c>
     </row>
-    <row r="190" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A190" s="5" t="s">
         <v>475</v>
       </c>
@@ -11196,7 +11200,7 @@
         <v>1031</v>
       </c>
     </row>
-    <row r="191" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A191" s="8" t="s">
         <v>477</v>
       </c>
@@ -11224,7 +11228,7 @@
         <v>1032</v>
       </c>
     </row>
-    <row r="192" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A192" s="5" t="s">
         <v>479</v>
       </c>
@@ -11252,7 +11256,7 @@
         <v>1033</v>
       </c>
     </row>
-    <row r="193" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A193" s="8" t="s">
         <v>481</v>
       </c>
@@ -11280,7 +11284,7 @@
         <v>1034</v>
       </c>
     </row>
-    <row r="194" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A194" s="5" t="s">
         <v>483</v>
       </c>
@@ -11308,7 +11312,7 @@
         <v>1035</v>
       </c>
     </row>
-    <row r="195" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A195" s="8" t="s">
         <v>485</v>
       </c>
@@ -11336,7 +11340,7 @@
         <v>1036</v>
       </c>
     </row>
-    <row r="196" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A196" s="5" t="s">
         <v>487</v>
       </c>
@@ -11364,7 +11368,7 @@
         <v>1037</v>
       </c>
     </row>
-    <row r="197" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A197" s="8" t="s">
         <v>489</v>
       </c>
@@ -11392,7 +11396,7 @@
         <v>1038</v>
       </c>
     </row>
-    <row r="198" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A198" s="5" t="s">
         <v>491</v>
       </c>
@@ -11420,7 +11424,7 @@
         <v>1039</v>
       </c>
     </row>
-    <row r="199" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A199" s="8" t="s">
         <v>493</v>
       </c>
@@ -11448,7 +11452,7 @@
         <v>1040</v>
       </c>
     </row>
-    <row r="200" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A200" s="5" t="s">
         <v>495</v>
       </c>
@@ -11476,7 +11480,7 @@
         <v>1041</v>
       </c>
     </row>
-    <row r="201" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A201" s="8" t="s">
         <v>497</v>
       </c>
@@ -11504,7 +11508,7 @@
         <v>1042</v>
       </c>
     </row>
-    <row r="202" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A202" s="5" t="s">
         <v>499</v>
       </c>
@@ -11532,7 +11536,7 @@
         <v>1043</v>
       </c>
     </row>
-    <row r="203" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A203" s="8" t="s">
         <v>501</v>
       </c>
@@ -11560,7 +11564,7 @@
         <v>1044</v>
       </c>
     </row>
-    <row r="204" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A204" s="5" t="s">
         <v>503</v>
       </c>
@@ -11588,7 +11592,7 @@
         <v>1045</v>
       </c>
     </row>
-    <row r="205" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A205" s="8" t="s">
         <v>505</v>
       </c>
@@ -11616,7 +11620,7 @@
         <v>1046</v>
       </c>
     </row>
-    <row r="206" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A206" s="5" t="s">
         <v>507</v>
       </c>
@@ -11644,7 +11648,7 @@
         <v>1047</v>
       </c>
     </row>
-    <row r="207" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A207" s="8" t="s">
         <v>509</v>
       </c>
@@ -11672,7 +11676,7 @@
         <v>1048</v>
       </c>
     </row>
-    <row r="208" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A208" s="5" t="s">
         <v>511</v>
       </c>
@@ -11700,7 +11704,7 @@
         <v>1049</v>
       </c>
     </row>
-    <row r="209" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A209" s="8" t="s">
         <v>513</v>
       </c>
@@ -11728,7 +11732,7 @@
         <v>1050</v>
       </c>
     </row>
-    <row r="210" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A210" s="5" t="s">
         <v>515</v>
       </c>
@@ -11756,7 +11760,7 @@
         <v>1051</v>
       </c>
     </row>
-    <row r="211" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A211" s="8" t="s">
         <v>517</v>
       </c>
@@ -11784,7 +11788,7 @@
         <v>1052</v>
       </c>
     </row>
-    <row r="212" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A212" s="5" t="s">
         <v>519</v>
       </c>
@@ -11812,7 +11816,7 @@
         <v>1053</v>
       </c>
     </row>
-    <row r="213" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A213" s="8" t="s">
         <v>521</v>
       </c>
@@ -11840,7 +11844,7 @@
         <v>1054</v>
       </c>
     </row>
-    <row r="214" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A214" s="5" t="s">
         <v>523</v>
       </c>
@@ -11868,7 +11872,7 @@
         <v>1055</v>
       </c>
     </row>
-    <row r="215" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A215" s="8" t="s">
         <v>525</v>
       </c>
@@ -11896,7 +11900,7 @@
         <v>1056</v>
       </c>
     </row>
-    <row r="216" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A216" s="5" t="s">
         <v>527</v>
       </c>
@@ -11924,7 +11928,7 @@
         <v>1057</v>
       </c>
     </row>
-    <row r="217" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A217" s="8" t="s">
         <v>529</v>
       </c>
@@ -11952,7 +11956,7 @@
         <v>1058</v>
       </c>
     </row>
-    <row r="218" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A218" s="5" t="s">
         <v>531</v>
       </c>
@@ -11980,7 +11984,7 @@
         <v>1059</v>
       </c>
     </row>
-    <row r="219" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A219" s="8" t="s">
         <v>533</v>
       </c>
@@ -12008,7 +12012,7 @@
         <v>1060</v>
       </c>
     </row>
-    <row r="220" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A220" s="5" t="s">
         <v>535</v>
       </c>
@@ -12036,7 +12040,7 @@
         <v>1061</v>
       </c>
     </row>
-    <row r="221" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A221" s="8" t="s">
         <v>537</v>
       </c>
@@ -12064,7 +12068,7 @@
         <v>1062</v>
       </c>
     </row>
-    <row r="222" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A222" s="5" t="s">
         <v>539</v>
       </c>
@@ -12092,7 +12096,7 @@
         <v>1063</v>
       </c>
     </row>
-    <row r="223" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A223" s="8" t="s">
         <v>541</v>
       </c>
@@ -12120,7 +12124,7 @@
         <v>1064</v>
       </c>
     </row>
-    <row r="224" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A224" s="5" t="s">
         <v>543</v>
       </c>
@@ -12148,7 +12152,7 @@
         <v>1065</v>
       </c>
     </row>
-    <row r="225" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A225" s="8" t="s">
         <v>545</v>
       </c>
@@ -12176,7 +12180,7 @@
         <v>1066</v>
       </c>
     </row>
-    <row r="226" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A226" s="5" t="s">
         <v>547</v>
       </c>
@@ -12204,7 +12208,7 @@
         <v>1067</v>
       </c>
     </row>
-    <row r="227" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A227" s="8" t="s">
         <v>549</v>
       </c>
@@ -12232,7 +12236,7 @@
         <v>1068</v>
       </c>
     </row>
-    <row r="228" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A228" s="5" t="s">
         <v>551</v>
       </c>
@@ -12260,7 +12264,7 @@
         <v>1069</v>
       </c>
     </row>
-    <row r="229" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A229" s="8" t="s">
         <v>553</v>
       </c>
@@ -12288,7 +12292,7 @@
         <v>1070</v>
       </c>
     </row>
-    <row r="230" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A230" s="5" t="s">
         <v>555</v>
       </c>
@@ -12316,7 +12320,7 @@
         <v>1071</v>
       </c>
     </row>
-    <row r="231" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A231" s="8" t="s">
         <v>557</v>
       </c>
@@ -12344,7 +12348,7 @@
         <v>1072</v>
       </c>
     </row>
-    <row r="232" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A232" s="5" t="s">
         <v>559</v>
       </c>
@@ -12372,7 +12376,7 @@
         <v>1073</v>
       </c>
     </row>
-    <row r="233" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A233" s="8" t="s">
         <v>561</v>
       </c>
@@ -12400,7 +12404,7 @@
         <v>1074</v>
       </c>
     </row>
-    <row r="234" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A234" s="5" t="s">
         <v>563</v>
       </c>
@@ -12428,7 +12432,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="235" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A235" s="8" t="s">
         <v>565</v>
       </c>
@@ -12456,7 +12460,7 @@
         <v>1076</v>
       </c>
     </row>
-    <row r="236" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A236" s="5" t="s">
         <v>567</v>
       </c>
@@ -12484,7 +12488,7 @@
         <v>1077</v>
       </c>
     </row>
-    <row r="237" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A237" s="8" t="s">
         <v>569</v>
       </c>
@@ -12512,7 +12516,7 @@
         <v>1078</v>
       </c>
     </row>
-    <row r="238" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A238" s="5" t="s">
         <v>571</v>
       </c>
@@ -12540,7 +12544,7 @@
         <v>1079</v>
       </c>
     </row>
-    <row r="239" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A239" s="8" t="s">
         <v>573</v>
       </c>
@@ -12568,7 +12572,7 @@
         <v>1080</v>
       </c>
     </row>
-    <row r="240" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A240" s="5" t="s">
         <v>575</v>
       </c>
@@ -12596,7 +12600,7 @@
         <v>1081</v>
       </c>
     </row>
-    <row r="241" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A241" s="8" t="s">
         <v>577</v>
       </c>
@@ -12624,7 +12628,7 @@
         <v>1082</v>
       </c>
     </row>
-    <row r="242" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A242" s="5" t="s">
         <v>579</v>
       </c>
@@ -12652,7 +12656,7 @@
         <v>1083</v>
       </c>
     </row>
-    <row r="243" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A243" s="8" t="s">
         <v>581</v>
       </c>
@@ -12680,7 +12684,7 @@
         <v>1084</v>
       </c>
     </row>
-    <row r="244" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A244" s="5" t="s">
         <v>583</v>
       </c>
@@ -12708,7 +12712,7 @@
         <v>1085</v>
       </c>
     </row>
-    <row r="245" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A245" s="8" t="s">
         <v>585</v>
       </c>
@@ -12736,7 +12740,7 @@
         <v>1086</v>
       </c>
     </row>
-    <row r="246" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A246" s="5" t="s">
         <v>587</v>
       </c>
@@ -12764,7 +12768,7 @@
         <v>1087</v>
       </c>
     </row>
-    <row r="247" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A247" s="8" t="s">
         <v>589</v>
       </c>
@@ -12792,7 +12796,7 @@
         <v>1088</v>
       </c>
     </row>
-    <row r="248" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A248" s="5" t="s">
         <v>591</v>
       </c>
@@ -12820,7 +12824,7 @@
         <v>1089</v>
       </c>
     </row>
-    <row r="249" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A249" s="8" t="s">
         <v>593</v>
       </c>
@@ -12848,7 +12852,7 @@
         <v>1090</v>
       </c>
     </row>
-    <row r="250" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A250" s="5" t="s">
         <v>595</v>
       </c>
@@ -12876,7 +12880,7 @@
         <v>1091</v>
       </c>
     </row>
-    <row r="251" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A251" s="8" t="s">
         <v>597</v>
       </c>
@@ -12904,7 +12908,7 @@
         <v>1092</v>
       </c>
     </row>
-    <row r="252" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A252" s="5" t="s">
         <v>599</v>
       </c>
@@ -12932,1237 +12936,1237 @@
         <v>1093</v>
       </c>
     </row>
-    <row r="253" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:43" x14ac:dyDescent="0.2">
       <c r="AQ253" s="10" t="s">
         <v>1094</v>
       </c>
     </row>
-    <row r="254" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:43" x14ac:dyDescent="0.2">
       <c r="AQ254" s="10" t="s">
         <v>1095</v>
       </c>
     </row>
-    <row r="255" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:43" x14ac:dyDescent="0.2">
       <c r="AQ255" s="10" t="s">
         <v>1096</v>
       </c>
     </row>
-    <row r="256" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:43" x14ac:dyDescent="0.2">
       <c r="AQ256" s="10" t="s">
         <v>1097</v>
       </c>
     </row>
-    <row r="257" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="257" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ257" s="10" t="s">
         <v>1098</v>
       </c>
     </row>
-    <row r="258" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="258" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ258" s="10" t="s">
         <v>1099</v>
       </c>
     </row>
-    <row r="259" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="259" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ259" s="10" t="s">
         <v>1100</v>
       </c>
     </row>
-    <row r="260" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="260" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ260" s="10" t="s">
         <v>1101</v>
       </c>
     </row>
-    <row r="261" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="261" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ261" s="10" t="s">
         <v>1102</v>
       </c>
     </row>
-    <row r="262" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="262" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ262" s="10" t="s">
         <v>1103</v>
       </c>
     </row>
-    <row r="263" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="263" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ263" s="10" t="s">
         <v>1104</v>
       </c>
     </row>
-    <row r="264" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="264" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ264" s="10" t="s">
         <v>1105</v>
       </c>
     </row>
-    <row r="265" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="265" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ265" s="10" t="s">
         <v>1106</v>
       </c>
     </row>
-    <row r="266" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="266" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ266" s="10" t="s">
         <v>1107</v>
       </c>
     </row>
-    <row r="267" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="267" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ267" s="10" t="s">
         <v>1108</v>
       </c>
     </row>
-    <row r="268" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="268" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ268" s="10" t="s">
         <v>1109</v>
       </c>
     </row>
-    <row r="269" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="269" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ269" s="10" t="s">
         <v>1110</v>
       </c>
     </row>
-    <row r="270" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="270" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ270" s="10" t="s">
         <v>1111</v>
       </c>
     </row>
-    <row r="271" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="271" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ271" s="10" t="s">
         <v>1112</v>
       </c>
     </row>
-    <row r="272" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="272" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ272" s="10" t="s">
         <v>1113</v>
       </c>
     </row>
-    <row r="273" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="273" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ273" s="10" t="s">
         <v>1114</v>
       </c>
     </row>
-    <row r="274" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="274" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ274" s="10" t="s">
         <v>1115</v>
       </c>
     </row>
-    <row r="275" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="275" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ275" s="10" t="s">
         <v>1116</v>
       </c>
     </row>
-    <row r="276" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="276" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ276" s="10" t="s">
         <v>1117</v>
       </c>
     </row>
-    <row r="277" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="277" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ277" s="10" t="s">
         <v>1118</v>
       </c>
     </row>
-    <row r="278" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="278" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ278" s="10" t="s">
         <v>1119</v>
       </c>
     </row>
-    <row r="279" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="279" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ279" s="10" t="s">
         <v>1120</v>
       </c>
     </row>
-    <row r="280" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="280" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ280" s="10" t="s">
         <v>1121</v>
       </c>
     </row>
-    <row r="281" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="281" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ281" s="10" t="s">
         <v>1122</v>
       </c>
     </row>
-    <row r="282" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="282" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ282" s="10" t="s">
         <v>1123</v>
       </c>
     </row>
-    <row r="283" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="283" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ283" t="s">
         <v>1124</v>
       </c>
     </row>
-    <row r="284" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="284" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ284" t="s">
         <v>1125</v>
       </c>
     </row>
-    <row r="285" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="285" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ285" s="10" t="s">
         <v>1126</v>
       </c>
     </row>
-    <row r="286" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="286" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ286" t="s">
         <v>1127</v>
       </c>
     </row>
-    <row r="287" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="287" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ287" t="s">
         <v>1128</v>
       </c>
     </row>
-    <row r="288" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="288" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ288" t="s">
         <v>1129</v>
       </c>
     </row>
-    <row r="289" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="289" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ289" t="s">
         <v>1130</v>
       </c>
     </row>
-    <row r="290" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="290" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ290" t="s">
         <v>1131</v>
       </c>
     </row>
-    <row r="291" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="291" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ291" t="s">
         <v>1132</v>
       </c>
     </row>
-    <row r="292" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="292" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ292" s="10" t="s">
         <v>1133</v>
       </c>
     </row>
-    <row r="293" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="293" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ293" s="10" t="s">
         <v>1134</v>
       </c>
     </row>
-    <row r="294" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="294" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ294" s="10" t="s">
         <v>1135</v>
       </c>
     </row>
-    <row r="295" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="295" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ295" s="10" t="s">
         <v>1136</v>
       </c>
     </row>
-    <row r="296" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="296" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ296" t="s">
         <v>1137</v>
       </c>
     </row>
-    <row r="297" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="297" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ297" t="s">
         <v>1138</v>
       </c>
     </row>
-    <row r="298" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="298" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ298" t="s">
         <v>1139</v>
       </c>
     </row>
-    <row r="299" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="299" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ299" t="s">
         <v>1140</v>
       </c>
     </row>
-    <row r="300" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="300" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ300" t="s">
         <v>1141</v>
       </c>
     </row>
-    <row r="301" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="301" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ301" t="s">
         <v>1142</v>
       </c>
     </row>
-    <row r="302" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="302" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ302" t="s">
         <v>1143</v>
       </c>
     </row>
-    <row r="303" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="303" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ303" t="s">
         <v>1144</v>
       </c>
     </row>
-    <row r="304" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="304" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ304" t="s">
         <v>1145</v>
       </c>
     </row>
-    <row r="305" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="305" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ305" t="s">
         <v>1146</v>
       </c>
     </row>
-    <row r="306" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="306" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ306" t="s">
         <v>1147</v>
       </c>
     </row>
-    <row r="307" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="307" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ307" t="s">
         <v>1148</v>
       </c>
     </row>
-    <row r="308" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="308" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ308" t="s">
         <v>1149</v>
       </c>
     </row>
-    <row r="309" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="309" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ309" t="s">
         <v>1150</v>
       </c>
     </row>
-    <row r="310" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="310" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ310" t="s">
         <v>1151</v>
       </c>
     </row>
-    <row r="311" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="311" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ311" t="s">
         <v>1152</v>
       </c>
     </row>
-    <row r="312" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="312" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ312" t="s">
         <v>1153</v>
       </c>
     </row>
-    <row r="313" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="313" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ313" t="s">
         <v>1154</v>
       </c>
     </row>
-    <row r="314" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="314" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ314" t="s">
         <v>1155</v>
       </c>
     </row>
-    <row r="315" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="315" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ315" t="s">
         <v>1156</v>
       </c>
     </row>
-    <row r="316" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="316" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ316" t="s">
         <v>1157</v>
       </c>
     </row>
-    <row r="317" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="317" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ317" s="10" t="s">
         <v>1158</v>
       </c>
     </row>
-    <row r="318" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="318" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ318" s="10" t="s">
         <v>1159</v>
       </c>
     </row>
-    <row r="319" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="319" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ319" s="10" t="s">
         <v>1160</v>
       </c>
     </row>
-    <row r="320" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="320" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ320" s="10" t="s">
         <v>1161</v>
       </c>
     </row>
-    <row r="321" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="321" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ321" s="10" t="s">
         <v>1162</v>
       </c>
     </row>
-    <row r="322" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="322" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ322" s="10" t="s">
         <v>1163</v>
       </c>
     </row>
-    <row r="323" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="323" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ323" s="10" t="s">
         <v>1164</v>
       </c>
     </row>
-    <row r="324" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="324" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ324" s="10" t="s">
         <v>1165</v>
       </c>
     </row>
-    <row r="325" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="325" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ325" s="10" t="s">
         <v>1166</v>
       </c>
     </row>
-    <row r="326" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="326" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ326" s="10" t="s">
         <v>1167</v>
       </c>
     </row>
-    <row r="327" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="327" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ327" s="10" t="s">
         <v>1168</v>
       </c>
     </row>
-    <row r="328" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="328" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ328" s="10" t="s">
         <v>1169</v>
       </c>
     </row>
-    <row r="329" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="329" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ329" s="10" t="s">
         <v>1170</v>
       </c>
     </row>
-    <row r="330" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="330" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ330" s="10" t="s">
         <v>1171</v>
       </c>
     </row>
-    <row r="331" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="331" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ331" s="10" t="s">
         <v>1172</v>
       </c>
     </row>
-    <row r="332" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="332" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ332" s="10" t="s">
         <v>1173</v>
       </c>
     </row>
-    <row r="333" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="333" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ333" s="10" t="s">
         <v>1174</v>
       </c>
     </row>
-    <row r="334" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="334" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ334" s="10" t="s">
         <v>1175</v>
       </c>
     </row>
-    <row r="335" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="335" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ335" s="10" t="s">
         <v>1176</v>
       </c>
     </row>
-    <row r="336" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="336" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ336" s="10" t="s">
         <v>1177</v>
       </c>
     </row>
-    <row r="337" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="337" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ337" s="10" t="s">
         <v>1178</v>
       </c>
     </row>
-    <row r="338" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="338" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ338" s="10" t="s">
         <v>1179</v>
       </c>
     </row>
-    <row r="339" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="339" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ339" s="10" t="s">
         <v>1180</v>
       </c>
     </row>
-    <row r="340" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="340" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ340" s="10" t="s">
         <v>1181</v>
       </c>
     </row>
-    <row r="341" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="341" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ341" s="10" t="s">
         <v>1182</v>
       </c>
     </row>
-    <row r="342" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="342" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ342" s="10" t="s">
         <v>1183</v>
       </c>
     </row>
-    <row r="343" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="343" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ343" s="10" t="s">
         <v>1184</v>
       </c>
     </row>
-    <row r="344" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="344" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ344" s="10" t="s">
         <v>1185</v>
       </c>
     </row>
-    <row r="345" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="345" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ345" s="10" t="s">
         <v>1186</v>
       </c>
     </row>
-    <row r="346" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="346" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ346" s="10" t="s">
         <v>1187</v>
       </c>
     </row>
-    <row r="347" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="347" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ347" s="10" t="s">
         <v>1188</v>
       </c>
     </row>
-    <row r="348" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="348" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ348" s="10" t="s">
         <v>1189</v>
       </c>
     </row>
-    <row r="349" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="349" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ349" s="10" t="s">
         <v>1190</v>
       </c>
     </row>
-    <row r="350" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="350" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ350" s="10" t="s">
         <v>1191</v>
       </c>
     </row>
-    <row r="351" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="351" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ351" s="10" t="s">
         <v>1192</v>
       </c>
     </row>
-    <row r="352" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="352" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ352" s="10" t="s">
         <v>1193</v>
       </c>
     </row>
-    <row r="353" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="353" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ353" s="10" t="s">
         <v>1194</v>
       </c>
     </row>
-    <row r="354" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="354" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ354" s="10" t="s">
         <v>1195</v>
       </c>
     </row>
-    <row r="355" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="355" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ355" s="10" t="s">
         <v>1196</v>
       </c>
     </row>
-    <row r="356" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="356" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ356" s="10" t="s">
         <v>1197</v>
       </c>
     </row>
-    <row r="357" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="357" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ357" s="10" t="s">
         <v>1198</v>
       </c>
     </row>
-    <row r="358" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="358" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ358" s="10" t="s">
         <v>1199</v>
       </c>
     </row>
-    <row r="359" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="359" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ359" s="10" t="s">
         <v>1200</v>
       </c>
     </row>
-    <row r="360" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="360" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ360" s="10" t="s">
         <v>1201</v>
       </c>
     </row>
-    <row r="361" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="361" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ361" s="10" t="s">
         <v>1202</v>
       </c>
     </row>
-    <row r="362" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="362" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ362" s="10" t="s">
         <v>1203</v>
       </c>
     </row>
-    <row r="363" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="363" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ363" s="10" t="s">
         <v>1204</v>
       </c>
     </row>
-    <row r="364" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="364" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ364" s="10" t="s">
         <v>1205</v>
       </c>
     </row>
-    <row r="365" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="365" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ365" s="10" t="s">
         <v>1206</v>
       </c>
     </row>
-    <row r="366" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="366" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ366" s="10" t="s">
         <v>1207</v>
       </c>
     </row>
-    <row r="367" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="367" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ367" s="10" t="s">
         <v>1208</v>
       </c>
     </row>
-    <row r="368" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="368" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ368" s="10" t="s">
         <v>1209</v>
       </c>
     </row>
-    <row r="369" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="369" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ369" s="10" t="s">
         <v>1210</v>
       </c>
     </row>
-    <row r="370" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="370" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ370" s="10" t="s">
         <v>1211</v>
       </c>
     </row>
-    <row r="371" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="371" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ371" s="10" t="s">
         <v>1212</v>
       </c>
     </row>
-    <row r="372" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="372" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ372" s="10" t="s">
         <v>1213</v>
       </c>
     </row>
-    <row r="373" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="373" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ373" s="10" t="s">
         <v>1214</v>
       </c>
     </row>
-    <row r="374" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="374" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ374" s="10" t="s">
         <v>1215</v>
       </c>
     </row>
-    <row r="375" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="375" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ375" s="10" t="s">
         <v>1216</v>
       </c>
     </row>
-    <row r="376" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="376" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ376" s="10" t="s">
         <v>1217</v>
       </c>
     </row>
-    <row r="377" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="377" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ377" s="10" t="s">
         <v>1218</v>
       </c>
     </row>
-    <row r="378" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="378" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ378" s="10" t="s">
         <v>1219</v>
       </c>
     </row>
-    <row r="379" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="379" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ379" s="10" t="s">
         <v>1220</v>
       </c>
     </row>
-    <row r="380" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="380" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ380" s="10" t="s">
         <v>1221</v>
       </c>
     </row>
-    <row r="381" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="381" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ381" s="10" t="s">
         <v>1222</v>
       </c>
     </row>
-    <row r="382" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="382" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ382" s="10" t="s">
         <v>1223</v>
       </c>
     </row>
-    <row r="383" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="383" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ383" s="10" t="s">
         <v>1224</v>
       </c>
     </row>
-    <row r="384" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="384" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ384" s="10" t="s">
         <v>1225</v>
       </c>
     </row>
-    <row r="385" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="385" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ385" s="10" t="s">
         <v>1226</v>
       </c>
     </row>
-    <row r="386" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="386" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ386" s="10" t="s">
         <v>1227</v>
       </c>
     </row>
-    <row r="387" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="387" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ387" s="10" t="s">
         <v>1228</v>
       </c>
     </row>
-    <row r="388" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="388" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ388" s="10" t="s">
         <v>1229</v>
       </c>
     </row>
-    <row r="389" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="389" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ389" s="10" t="s">
         <v>1230</v>
       </c>
     </row>
-    <row r="390" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="390" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ390" s="10" t="s">
         <v>1231</v>
       </c>
     </row>
-    <row r="391" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="391" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ391" s="10" t="s">
         <v>1232</v>
       </c>
     </row>
-    <row r="392" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="392" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ392" s="10" t="s">
         <v>1233</v>
       </c>
     </row>
-    <row r="393" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="393" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ393" s="10" t="s">
         <v>1234</v>
       </c>
     </row>
-    <row r="394" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="394" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ394" s="10" t="s">
         <v>1235</v>
       </c>
     </row>
-    <row r="395" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="395" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ395" s="10" t="s">
         <v>1236</v>
       </c>
     </row>
-    <row r="396" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="396" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ396" s="10" t="s">
         <v>1237</v>
       </c>
     </row>
-    <row r="397" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="397" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ397" s="10" t="s">
         <v>1238</v>
       </c>
     </row>
-    <row r="398" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="398" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ398" s="10" t="s">
         <v>1239</v>
       </c>
     </row>
-    <row r="399" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="399" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ399" s="10" t="s">
         <v>1240</v>
       </c>
     </row>
-    <row r="400" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="400" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ400" s="10" t="s">
         <v>1241</v>
       </c>
     </row>
-    <row r="401" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="401" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ401" s="10" t="s">
         <v>1242</v>
       </c>
     </row>
-    <row r="402" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="402" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ402" s="10" t="s">
         <v>1243</v>
       </c>
     </row>
-    <row r="403" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="403" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ403" s="10" t="s">
         <v>1244</v>
       </c>
     </row>
-    <row r="404" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="404" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ404" s="10" t="s">
         <v>1245</v>
       </c>
     </row>
-    <row r="405" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="405" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ405" s="10" t="s">
         <v>1246</v>
       </c>
     </row>
-    <row r="406" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="406" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ406" s="10" t="s">
         <v>1247</v>
       </c>
     </row>
-    <row r="407" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="407" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ407" s="10" t="s">
         <v>1248</v>
       </c>
     </row>
-    <row r="408" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="408" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ408" s="10" t="s">
         <v>1249</v>
       </c>
     </row>
-    <row r="409" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="409" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ409" s="10" t="s">
         <v>1250</v>
       </c>
     </row>
-    <row r="410" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="410" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ410" s="10" t="s">
         <v>1251</v>
       </c>
     </row>
-    <row r="411" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="411" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ411" s="10" t="s">
         <v>1252</v>
       </c>
     </row>
-    <row r="412" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="412" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ412" s="10" t="s">
         <v>1253</v>
       </c>
     </row>
-    <row r="413" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="413" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ413" s="10" t="s">
         <v>1254</v>
       </c>
     </row>
-    <row r="414" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="414" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ414" s="10" t="s">
         <v>1255</v>
       </c>
     </row>
-    <row r="415" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="415" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ415" s="10" t="s">
         <v>1256</v>
       </c>
     </row>
-    <row r="416" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="416" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ416" s="10" t="s">
         <v>1257</v>
       </c>
     </row>
-    <row r="417" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="417" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ417" t="s">
         <v>1258</v>
       </c>
     </row>
-    <row r="418" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="418" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ418" t="s">
         <v>1259</v>
       </c>
     </row>
-    <row r="419" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="419" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ419" t="s">
         <v>1260</v>
       </c>
     </row>
-    <row r="420" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="420" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ420" t="s">
         <v>1261</v>
       </c>
     </row>
-    <row r="421" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="421" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ421" t="s">
         <v>1262</v>
       </c>
     </row>
-    <row r="422" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="422" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ422" t="s">
         <v>1263</v>
       </c>
     </row>
-    <row r="423" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="423" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ423" t="s">
         <v>1264</v>
       </c>
     </row>
-    <row r="424" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="424" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ424" t="s">
         <v>1265</v>
       </c>
     </row>
-    <row r="425" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="425" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ425" t="s">
         <v>1266</v>
       </c>
     </row>
-    <row r="426" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="426" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ426" t="s">
         <v>1267</v>
       </c>
     </row>
-    <row r="427" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="427" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ427" t="s">
         <v>1268</v>
       </c>
     </row>
-    <row r="428" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="428" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ428" t="s">
         <v>1269</v>
       </c>
     </row>
-    <row r="429" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="429" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ429" t="s">
         <v>1270</v>
       </c>
     </row>
-    <row r="430" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="430" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ430" t="s">
         <v>1271</v>
       </c>
     </row>
-    <row r="431" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="431" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ431" t="s">
         <v>1272</v>
       </c>
     </row>
-    <row r="432" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="432" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ432" s="10" t="s">
         <v>1273</v>
       </c>
     </row>
-    <row r="433" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="433" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ433" s="10" t="s">
         <v>1274</v>
       </c>
     </row>
-    <row r="434" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="434" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ434" s="10" t="s">
         <v>1275</v>
       </c>
     </row>
-    <row r="435" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="435" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ435" s="10" t="s">
         <v>1276</v>
       </c>
     </row>
-    <row r="436" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="436" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ436" s="10" t="s">
         <v>1277</v>
       </c>
     </row>
-    <row r="437" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="437" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ437" s="10" t="s">
         <v>1278</v>
       </c>
     </row>
-    <row r="438" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="438" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ438" s="10" t="s">
         <v>1279</v>
       </c>
     </row>
-    <row r="439" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="439" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ439" s="10" t="s">
         <v>1280</v>
       </c>
     </row>
-    <row r="440" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="440" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ440" s="10" t="s">
         <v>1281</v>
       </c>
     </row>
-    <row r="441" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="441" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ441" s="10" t="s">
         <v>1282</v>
       </c>
     </row>
-    <row r="442" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="442" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ442" s="10" t="s">
         <v>1283</v>
       </c>
     </row>
-    <row r="443" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="443" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ443" s="10" t="s">
         <v>1284</v>
       </c>
     </row>
-    <row r="444" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="444" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ444" s="10" t="s">
         <v>1285</v>
       </c>
     </row>
-    <row r="445" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="445" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ445" s="10" t="s">
         <v>1286</v>
       </c>
     </row>
-    <row r="446" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="446" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ446" s="10" t="s">
         <v>1287</v>
       </c>
     </row>
-    <row r="447" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="447" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ447" s="10" t="s">
         <v>1288</v>
       </c>
     </row>
-    <row r="448" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="448" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ448" s="10" t="s">
         <v>1289</v>
       </c>
     </row>
-    <row r="449" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="449" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ449" s="10" t="s">
         <v>1290</v>
       </c>
     </row>
-    <row r="450" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="450" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ450" s="10" t="s">
         <v>1291</v>
       </c>
     </row>
-    <row r="451" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="451" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ451" s="10" t="s">
         <v>1292</v>
       </c>
     </row>
-    <row r="452" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="452" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ452" s="10" t="s">
         <v>1293</v>
       </c>
     </row>
-    <row r="453" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="453" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ453" s="10" t="s">
         <v>1294</v>
       </c>
     </row>
-    <row r="454" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="454" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ454" s="10" t="s">
         <v>1295</v>
       </c>
     </row>
-    <row r="455" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="455" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ455" s="10" t="s">
         <v>1296</v>
       </c>
     </row>
-    <row r="456" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="456" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ456" s="10" t="s">
         <v>1297</v>
       </c>
     </row>
-    <row r="457" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="457" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ457" s="10" t="s">
         <v>1298</v>
       </c>
     </row>
-    <row r="458" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="458" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ458" s="10" t="s">
         <v>1299</v>
       </c>
     </row>
-    <row r="459" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="459" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ459" s="10" t="s">
         <v>1300</v>
       </c>
     </row>
-    <row r="460" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="460" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ460" s="10" t="s">
         <v>1301</v>
       </c>
     </row>
-    <row r="461" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="461" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ461" s="10" t="s">
         <v>1302</v>
       </c>
     </row>
-    <row r="462" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="462" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ462" s="10" t="s">
         <v>1303</v>
       </c>
     </row>
-    <row r="463" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="463" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ463" s="10" t="s">
         <v>1304</v>
       </c>
     </row>
-    <row r="464" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="464" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ464" s="10" t="s">
         <v>1305</v>
       </c>
     </row>
-    <row r="465" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="465" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ465" s="10" t="s">
         <v>1306</v>
       </c>
     </row>
-    <row r="466" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="466" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ466" s="10" t="s">
         <v>1307</v>
       </c>
     </row>
-    <row r="467" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="467" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ467" s="10" t="s">
         <v>1308</v>
       </c>
     </row>
-    <row r="468" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="468" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ468" s="10" t="s">
         <v>1309</v>
       </c>
     </row>
-    <row r="469" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="469" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ469" s="10" t="s">
         <v>1310</v>
       </c>
     </row>
-    <row r="470" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="470" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ470" s="10" t="s">
         <v>1311</v>
       </c>
     </row>
-    <row r="471" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="471" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ471" s="10" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="472" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="472" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ472" s="10" t="s">
         <v>1313</v>
       </c>
     </row>
-    <row r="473" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="473" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ473" s="10" t="s">
         <v>1314</v>
       </c>
     </row>
-    <row r="474" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="474" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ474" s="10" t="s">
         <v>1315</v>
       </c>
     </row>
-    <row r="475" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="475" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ475" s="10" t="s">
         <v>1316</v>
       </c>
     </row>
-    <row r="476" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="476" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ476" s="10" t="s">
         <v>1317</v>
       </c>
     </row>
-    <row r="477" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="477" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ477" s="10" t="s">
         <v>1318</v>
       </c>
     </row>
-    <row r="478" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="478" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ478" s="10" t="s">
         <v>1319</v>
       </c>
     </row>
-    <row r="479" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="479" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ479" s="10" t="s">
         <v>1320</v>
       </c>
     </row>
-    <row r="480" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="480" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ480" t="s">
         <v>1321</v>
       </c>
     </row>
-    <row r="481" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="481" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ481" t="s">
         <v>1322</v>
       </c>
     </row>
-    <row r="482" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="482" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ482" t="s">
         <v>1323</v>
       </c>
     </row>
-    <row r="483" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="483" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ483" t="s">
         <v>1324</v>
       </c>
     </row>
-    <row r="484" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="484" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ484" t="s">
         <v>1325</v>
       </c>
     </row>
-    <row r="485" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="485" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ485" t="s">
         <v>1326</v>
       </c>
     </row>
-    <row r="486" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="486" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ486" t="s">
         <v>1327</v>
       </c>
     </row>
-    <row r="487" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="487" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ487" t="s">
         <v>1328</v>
       </c>
     </row>
-    <row r="488" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="488" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ488" t="s">
         <v>1329</v>
       </c>
     </row>
-    <row r="489" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="489" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ489" s="10" t="s">
         <v>1330</v>
       </c>
     </row>
-    <row r="490" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="490" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ490" t="s">
         <v>1331</v>
       </c>
     </row>
-    <row r="491" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="491" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ491" t="s">
         <v>1332</v>
       </c>
     </row>
-    <row r="492" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="492" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ492" s="10" t="s">
         <v>1333</v>
       </c>
     </row>
-    <row r="493" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="493" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ493" s="10" t="s">
         <v>1334</v>
       </c>
     </row>
-    <row r="494" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="494" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ494" s="10" t="s">
         <v>1335</v>
       </c>
     </row>
-    <row r="495" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="495" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ495" s="10" t="s">
         <v>1336</v>
       </c>
     </row>
-    <row r="496" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="496" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ496" s="10" t="s">
         <v>1337</v>
       </c>
     </row>
-    <row r="497" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="497" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ497" s="10" t="s">
         <v>1338</v>
       </c>
     </row>
-    <row r="498" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="498" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ498" s="10" t="s">
         <v>1339</v>
       </c>
     </row>
-    <row r="499" spans="43:43" x14ac:dyDescent="0.35">
+    <row r="499" spans="43:43" x14ac:dyDescent="0.2">
       <c r="AQ499" s="10" t="s">
         <v>1340</v>
       </c>

</xml_diff>